<commit_message>
auto commit: 2026-03-21 15:43:25
</commit_message>
<xml_diff>
--- a/快乐羊毛系统/功能测试需要的文件2026.03.17/UI自动化docs/测试用例/现有系统后台/后台_品牌管理.xlsx
+++ b/快乐羊毛系统/功能测试需要的文件2026.03.17/UI自动化docs/测试用例/现有系统后台/后台_品牌管理.xlsx
@@ -306,7 +306,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -325,13 +325,6 @@
       <sz val="10"/>
       <name val="微软雅黑"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <u/>
@@ -802,148 +795,148 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>

</xml_diff>

<commit_message>
auto commit: 2026-03-21 15:59:19
</commit_message>
<xml_diff>
--- a/快乐羊毛系统/功能测试需要的文件2026.03.17/UI自动化docs/测试用例/现有系统后台/后台_品牌管理.xlsx
+++ b/快乐羊毛系统/功能测试需要的文件2026.03.17/UI自动化docs/测试用例/现有系统后台/后台_品牌管理.xlsx
@@ -4,10 +4,11 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="11925"/>
+    <workbookView windowWidth="27945" windowHeight="11925" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="测试用例" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="82">
   <si>
     <t>用例编号</t>
   </si>
@@ -294,6 +295,12 @@
   <si>
     <t>1. 页面正常加载
 2. 支持轮播图的添加、编辑、删除、排序</t>
+  </si>
+  <si>
+    <t>用例标题</t>
+  </si>
+  <si>
+    <t>预期结果（断言）</t>
   </si>
 </sst>
 </file>
@@ -306,10 +313,23 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="24">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -671,7 +691,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -683,6 +703,32 @@
       <left style="thin">
         <color auto="1"/>
       </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="thin">
         <color auto="1"/>
       </right>
@@ -810,145 +856,166 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1309,364 +1376,466 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" spans="1:6">
+      <c r="A1" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" ht="82.5" spans="1:6">
+      <c r="A2" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" ht="82.5" spans="1:6">
+      <c r="A3" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" ht="33" spans="1:6">
+      <c r="A4" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" ht="49.5" spans="1:6">
+      <c r="A5" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="F5" s="10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" ht="49.5" spans="1:6">
+      <c r="A6" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="F6" s="10" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" ht="33" spans="1:6">
+      <c r="A7" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8" ht="33" spans="1:6">
+      <c r="A8" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="F8" s="10" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="9" ht="33" spans="1:6">
+      <c r="A9" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" ht="33" spans="1:6">
+      <c r="A10" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="F10" s="10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="11" ht="33" spans="1:6">
+      <c r="A11" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="F11" s="10" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="12" ht="33" spans="1:6">
+      <c r="A12" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="D12" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="E12" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="F12" s="10" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="13" ht="33" spans="1:6">
+      <c r="A13" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="D13" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="F13" s="10" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="14" ht="16.5" spans="1:6">
+      <c r="A14" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="D14" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="F14" s="10" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="15" ht="33" spans="1:6">
+      <c r="A15" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="F15" s="10" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="16" ht="33" spans="1:6">
+      <c r="A16" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C16" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="D16" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="E16" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="F16" s="10" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="17" ht="33" spans="1:6">
+      <c r="A17" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="F17" s="10" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="18" ht="33" spans="1:6">
+      <c r="A18" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="D18" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="E18" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="F18" s="10" t="s">
+        <v>79</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="4"/>
+  <cols>
+    <col min="1" max="5" width="12.875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>80</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" ht="82.5" spans="1:6">
-      <c r="A2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" ht="82.5" spans="1:6">
-      <c r="A3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" ht="33" spans="1:6">
-      <c r="A4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="5" ht="49.5" spans="1:6">
-      <c r="A5" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="6" ht="49.5" spans="1:6">
-      <c r="A6" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="7" ht="33" spans="1:6">
-      <c r="A7" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="8" ht="33" spans="1:6">
-      <c r="A8" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="9" ht="33" spans="1:6">
-      <c r="A9" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="10" ht="33" spans="1:6">
-      <c r="A10" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="11" ht="33" spans="1:6">
-      <c r="A11" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="12" ht="33" spans="1:6">
-      <c r="A12" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="13" ht="33" spans="1:6">
-      <c r="A13" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="14" ht="16.5" spans="1:6">
-      <c r="A14" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="15" ht="33" spans="1:6">
-      <c r="A15" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="16" ht="33" spans="1:6">
-      <c r="A16" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="17" ht="33" spans="1:6">
-      <c r="A17" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="18" ht="33" spans="1:6">
-      <c r="A18" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>79</v>
-      </c>
+      <c r="E1" s="2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" s="1"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="6"/>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" s="1"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="6"/>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="1"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="6"/>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" s="1"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="6"/>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" s="1"/>
+      <c r="B6" s="3"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="6"/>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" s="1"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="6"/>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" s="1"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="6"/>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" s="1"/>
+      <c r="B9" s="7"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" s="1"/>
+      <c r="B10" s="7"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" s="1"/>
+      <c r="B11" s="1"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>